<commit_message>
Nuovi prodotti, piani ALMAVIRIA, fix export CSV compensi
- Aggiunti Wind Tre FISSO, Edison Fix/Dynamic, Acea Trend, Plenitude Business
- Sky: gestoreId=33, fornitore De Iaco Service
- compOverride FEDERAZIENDE su Edison, Acea, Estra, Fastweb, Iren, AGN, Plenitude
- Magis: gettone ridotto del 22% (senza IVA)
- AFF FEDER = FEDERAZIENDE × 0.70, arrotondamento a decina/5
- ALMAVIRIA A = gettone × 0.68, ALMAVIRIA/B = gettone × 0.765 (non derivano da FEDER)
- Aggiunto piano ALMAVIRIA B
- Lion escluso da FEDERAZIENDE e AFF FEDER
- Fix export CSV: ora include tutti i gestori (es. A2A) rimosso skip errato
- Tipo TELECOM mostra tecnologia e canone nel nome prodotto

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Calcolatore_Completo_SM_AGN_Magis.xlsx
+++ b/Calcolatore_Completo_SM_AGN_Magis.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/debbypalazzogmail.com/Documents/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/debbypalazzogmail.com/Downloads/calcolocompensi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FE2D83D9-1614-1044-BA26-0C1A695AA77D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{351AB090-E5D3-F048-99A6-4B86471DBBD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="16380" windowHeight="16640" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -941,267 +941,267 @@
   </cellStyleXfs>
   <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="9" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="27" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="28" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="30" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="32" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="29" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="9" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="25" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="27" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="28" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="30" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="32" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1483,550 +1483,550 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="82" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
+      <c r="C2" s="82"/>
+      <c r="D2" s="82"/>
     </row>
     <row r="3" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="83" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
+      <c r="C3" s="83"/>
+      <c r="D3" s="83"/>
     </row>
     <row r="5" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="81" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="F5" s="15" t="s">
+      <c r="C5" s="81"/>
+      <c r="D5" s="81"/>
+      <c r="F5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="15" t="s">
+      <c r="G5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="H5" s="15" t="s">
+      <c r="H5" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F6" s="16" t="s">
+      <c r="F6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G6" s="17" t="s">
+      <c r="G6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H6" s="18">
+      <c r="H6" s="7">
         <v>95</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="20">
+      <c r="C7" s="9">
         <v>300</v>
       </c>
-      <c r="F7" s="21" t="s">
+      <c r="F7" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="22" t="s">
+      <c r="G7" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="H7" s="23">
+      <c r="H7" s="12">
         <v>80</v>
       </c>
     </row>
     <row r="8" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="C8" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="25">
+      <c r="D8" s="14">
         <f>IF(LEFT(C8,2)="E1",95,IF(LEFT(C8,2)="E2",80,55))</f>
         <v>80</v>
       </c>
-      <c r="F8" s="26" t="s">
+      <c r="F8" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="27" t="s">
+      <c r="G8" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H8" s="28">
+      <c r="H8" s="17">
         <v>55</v>
       </c>
     </row>
     <row r="9" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="25">
+      <c r="D9" s="14">
         <f>IF(RIGHT(C9,2)="€5",5,IF(RIGHT(C9,3)="€20",20,IF(RIGHT(C9,3)="€30",30,35)))</f>
         <v>35</v>
       </c>
     </row>
     <row r="10" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="24" t="s">
+      <c r="C10" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="29">
+      <c r="D10" s="18">
         <f>VALUE(SUBSTITUTE(C10,"%",""))/100</f>
         <v>0.75</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G10" s="15" t="s">
+      <c r="G10" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H10" s="15" t="s">
+      <c r="H10" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="11" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F11" s="30" t="s">
+      <c r="F11" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="G11" s="30" t="s">
+      <c r="G11" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="H11" s="31">
+      <c r="H11" s="20">
         <v>5</v>
       </c>
     </row>
     <row r="12" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="84" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="F12" s="32" t="s">
+      <c r="C12" s="84"/>
+      <c r="D12" s="84"/>
+      <c r="F12" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="G12" s="32" t="s">
+      <c r="G12" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="H12" s="33">
+      <c r="H12" s="22">
         <v>20</v>
       </c>
     </row>
     <row r="13" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="34" t="s">
+      <c r="B13" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="35" t="s">
+      <c r="C13" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="D13" s="36">
+      <c r="D13" s="25">
         <f>D8</f>
         <v>80</v>
       </c>
-      <c r="F13" s="30" t="s">
+      <c r="F13" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="G13" s="30" t="s">
+      <c r="G13" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="H13" s="31">
+      <c r="H13" s="20">
         <v>30</v>
       </c>
     </row>
     <row r="14" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="37" t="s">
+      <c r="B14" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="38" t="str">
+      <c r="C14" s="27" t="str">
         <f>"€"&amp;D9&amp;" x "&amp;TEXT(D10,"0%")</f>
         <v>€35 x 75%</v>
       </c>
-      <c r="D14" s="39">
+      <c r="D14" s="28">
         <f>D9*D10</f>
         <v>26.25</v>
       </c>
-      <c r="F14" s="32" t="s">
+      <c r="F14" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="G14" s="32" t="s">
+      <c r="G14" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="33">
+      <c r="H14" s="22">
         <v>35</v>
       </c>
     </row>
     <row r="15" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="40" t="s">
+      <c r="B15" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="41" t="str">
+      <c r="C15" s="30" t="str">
         <f>IF(C7&gt;500,"GOLD","ENTRY LEVEL")</f>
         <v>ENTRY LEVEL</v>
       </c>
-      <c r="D15" s="42">
+      <c r="D15" s="31">
         <f>IF(C7&lt;=500,IF(C7&gt;0,(MIN(C7,250)*5+MIN(MAX(C7-250,0),100)*14+MIN(MAX(C7-350,0),150)*18)/C7,0),IF(C7&gt;1500,30,IF(C7&gt;1000,20,10)))</f>
         <v>6.5</v>
       </c>
     </row>
     <row r="16" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F16" s="15" t="s">
+      <c r="F16" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="G16" s="15" t="s">
+      <c r="G16" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="H16" s="15" t="s">
+      <c r="H16" s="4" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="85" t="s">
         <v>24</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="43">
+      <c r="C17" s="85"/>
+      <c r="D17" s="32">
         <f>D13+D14+D15</f>
         <v>112.75</v>
       </c>
-      <c r="F17" s="27" t="s">
+      <c r="F17" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="G17" s="27" t="s">
+      <c r="G17" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="H17" s="28">
+      <c r="H17" s="17">
         <v>5</v>
       </c>
     </row>
     <row r="18" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F18" s="27" t="s">
+      <c r="F18" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="G18" s="27" t="s">
+      <c r="G18" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="H18" s="28">
+      <c r="H18" s="17">
         <v>14</v>
       </c>
     </row>
     <row r="19" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="77" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="F19" s="27" t="s">
+      <c r="C19" s="77"/>
+      <c r="D19" s="77"/>
+      <c r="F19" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="G19" s="27" t="s">
+      <c r="G19" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="H19" s="28">
+      <c r="H19" s="17">
         <v>18</v>
       </c>
     </row>
     <row r="20" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="45" t="s">
+      <c r="B20" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="46" t="s">
+      <c r="C20" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="D20" s="47">
+      <c r="D20" s="35">
         <f>ROUND(D17*0.01,2)</f>
         <v>1.1299999999999999</v>
       </c>
     </row>
     <row r="21" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="45" t="s">
+      <c r="B21" s="33" t="s">
         <v>42</v>
       </c>
-      <c r="C21" s="46" t="s">
+      <c r="C21" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="D21" s="47">
+      <c r="D21" s="35">
         <f>ROUND(D17*0.23*0.2,2)</f>
         <v>5.19</v>
       </c>
-      <c r="F21" s="48" t="s">
+      <c r="F21" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="G21" s="48" t="s">
+      <c r="G21" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="H21" s="48" t="s">
+      <c r="H21" s="2" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="45" t="s">
+      <c r="B22" s="33" t="s">
         <v>46</v>
       </c>
-      <c r="C22" s="46" t="str">
+      <c r="C22" s="34" t="str">
         <f>TEXT(D22/D17*100,"0.00")&amp;"% del lordo"</f>
         <v>006% del lordo</v>
       </c>
-      <c r="D22" s="47">
+      <c r="D22" s="35">
         <f>D20+D21</f>
         <v>6.32</v>
       </c>
-      <c r="F22" s="49" t="s">
+      <c r="F22" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="G22" s="49" t="s">
+      <c r="G22" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="H22" s="50">
+      <c r="H22" s="37">
         <v>10</v>
       </c>
     </row>
     <row r="23" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F23" s="49" t="s">
+      <c r="F23" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="G23" s="49" t="s">
+      <c r="G23" s="36" t="s">
         <v>49</v>
       </c>
-      <c r="H23" s="50">
+      <c r="H23" s="37">
         <v>20</v>
       </c>
     </row>
     <row r="24" spans="2:8" ht="64.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="78" t="s">
         <v>50</v>
       </c>
-      <c r="C24" s="8"/>
-      <c r="D24" s="51">
+      <c r="C24" s="78"/>
+      <c r="D24" s="38">
         <f>D17-D22</f>
         <v>106.43</v>
       </c>
-      <c r="F24" s="49" t="s">
+      <c r="F24" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="G24" s="49" t="s">
+      <c r="G24" s="36" t="s">
         <v>51</v>
       </c>
-      <c r="H24" s="50">
+      <c r="H24" s="37">
         <v>30</v>
       </c>
     </row>
     <row r="26" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="79" t="s">
         <v>52</v>
       </c>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="F26" s="15" t="s">
+      <c r="C26" s="79"/>
+      <c r="D26" s="79"/>
+      <c r="F26" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="G26" s="15"/>
-      <c r="H26" s="15" t="s">
+      <c r="G26" s="4"/>
+      <c r="H26" s="4" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="27" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="26" t="s">
+      <c r="B27" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="C27" s="27" t="str">
+      <c r="C27" s="16" t="str">
         <f>MIN(C7,250)&amp;" ctr"</f>
         <v>250 ctr</v>
       </c>
-      <c r="D27" s="52">
+      <c r="D27" s="39">
         <f>IF(C7&lt;=500,MIN(C7,250)*5,"-")</f>
         <v>1250</v>
       </c>
-      <c r="F27" s="53" t="s">
+      <c r="F27" s="40" t="s">
         <v>55</v>
       </c>
-      <c r="H27" s="54" t="s">
+      <c r="H27" s="41" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="28" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="26" t="s">
+      <c r="B28" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="C28" s="27" t="str">
+      <c r="C28" s="16" t="str">
         <f>MIN(MAX(C7-250,0),100)&amp;" ctr"</f>
         <v>50 ctr</v>
       </c>
-      <c r="D28" s="52">
+      <c r="D28" s="39">
         <f>IF(C7&lt;=500,MIN(MAX(C7-250,0),100)*14,"-")</f>
         <v>700</v>
       </c>
-      <c r="F28" s="53" t="s">
+      <c r="F28" s="40" t="s">
         <v>58</v>
       </c>
-      <c r="H28" s="54" t="s">
+      <c r="H28" s="41" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="29" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="26" t="s">
+      <c r="B29" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="C29" s="27" t="str">
+      <c r="C29" s="16" t="str">
         <f>MIN(MAX(C7-350,0),150)&amp;" ctr"</f>
         <v>0 ctr</v>
       </c>
-      <c r="D29" s="52">
+      <c r="D29" s="39">
         <f>IF(C7&lt;=500,MIN(MAX(C7-350,0),150)*18,"-")</f>
         <v>0</v>
       </c>
-      <c r="F29" s="45" t="s">
+      <c r="F29" s="33" t="s">
         <v>46</v>
       </c>
-      <c r="H29" s="55" t="s">
+      <c r="H29" s="42" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="30" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B30" s="19" t="s">
+      <c r="B30" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="D30" s="56">
+      <c r="D30" s="43">
         <f>IF(C7&lt;=500,IF(ISNUMBER(D27),D27,0)+IF(ISNUMBER(D28),D28,0)+IF(ISNUMBER(D29),D29,0),"-")</f>
         <v>1950</v>
       </c>
     </row>
     <row r="32" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="80" t="s">
         <v>63</v>
       </c>
-      <c r="C32" s="6"/>
-      <c r="D32" s="6"/>
+      <c r="C32" s="80"/>
+      <c r="D32" s="80"/>
     </row>
     <row r="33" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="57" t="s">
+      <c r="B33" s="44" t="s">
         <v>64</v>
       </c>
-      <c r="C33" s="49" t="str">
+      <c r="C33" s="36" t="str">
         <f>IF(C7&gt;500,C7&amp;" x €10","")</f>
         <v/>
       </c>
-      <c r="D33" s="58" t="str">
+      <c r="D33" s="45" t="str">
         <f>IF(C7&gt;500,IF(C7&lt;=1000,C7*10,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="34" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="57" t="s">
+      <c r="B34" s="44" t="s">
         <v>65</v>
       </c>
-      <c r="C34" s="49" t="str">
+      <c r="C34" s="36" t="str">
         <f>IF(C7&gt;1000,C7&amp;" x €20","")</f>
         <v/>
       </c>
-      <c r="D34" s="58" t="str">
+      <c r="D34" s="45" t="str">
         <f>IF(C7&gt;1000,IF(C7&lt;=1500,C7*20,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="35" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="57" t="s">
+      <c r="B35" s="44" t="s">
         <v>66</v>
       </c>
-      <c r="C35" s="49" t="str">
+      <c r="C35" s="36" t="str">
         <f>IF(C7&gt;1500,C7&amp;" x €30","")</f>
         <v/>
       </c>
-      <c r="D35" s="58" t="str">
+      <c r="D35" s="45" t="str">
         <f>IF(C7&gt;1500,C7*30,"")</f>
         <v/>
       </c>
     </row>
     <row r="36" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B36" s="57" t="s">
+      <c r="B36" s="44" t="s">
         <v>67</v>
       </c>
-      <c r="D36" s="59" t="str">
+      <c r="D36" s="46" t="str">
         <f>IF(C7&gt;500,IF(C7&lt;=1000,C7*10,IF(C7&lt;=1500,C7*20,C7*30)),"")</f>
         <v/>
       </c>
     </row>
     <row r="38" spans="2:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="12" t="s">
+      <c r="B38" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C38" s="12"/>
-      <c r="D38" s="12"/>
+      <c r="C38" s="81"/>
+      <c r="D38" s="81"/>
     </row>
     <row r="39" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="60" t="s">
+      <c r="B39" s="47" t="s">
         <v>69</v>
       </c>
-      <c r="D39" s="61">
+      <c r="D39" s="48">
         <f>C7*D8</f>
         <v>24000</v>
       </c>
     </row>
     <row r="40" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B40" s="60" t="s">
+      <c r="B40" s="47" t="s">
         <v>70</v>
       </c>
-      <c r="D40" s="61">
+      <c r="D40" s="48">
         <f>ROUND(C7*D10,0)*D9</f>
         <v>7875</v>
       </c>
     </row>
     <row r="41" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B41" s="60" t="s">
+      <c r="B41" s="47" t="s">
         <v>71</v>
       </c>
-      <c r="D41" s="61">
+      <c r="D41" s="48">
         <f>IF(C7&lt;=500,IF(ISNUMBER(D30),D30,0),IF(ISNUMBER(D36),D36,0))</f>
         <v>1950</v>
       </c>
     </row>
     <row r="42" spans="2:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B42" s="62" t="s">
+      <c r="B42" s="49" t="s">
         <v>72</v>
       </c>
-      <c r="D42" s="63">
+      <c r="D42" s="50">
         <f>D39+D40+D41</f>
         <v>33825</v>
       </c>
     </row>
     <row r="43" spans="2:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B43" s="53" t="s">
+      <c r="B43" s="40" t="s">
         <v>73</v>
       </c>
-      <c r="D43" s="64">
+      <c r="D43" s="51">
         <f>D42*0.01+ROUND(D42*0.23*0.2,0)</f>
         <v>1894.25</v>
       </c>
     </row>
     <row r="44" spans="2:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B44" s="65" t="s">
+      <c r="B44" s="52" t="s">
         <v>74</v>
       </c>
-      <c r="D44" s="66">
+      <c r="D44" s="53">
         <f>D42-D43</f>
         <v>31930.75</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B17:C17"/>
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B26:D26"/>
     <mergeCell ref="B32:D32"/>
     <mergeCell ref="B38:D38"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B17:C17"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation type="list" sqref="C8" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -2065,322 +2065,322 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="86" t="s">
         <v>75</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
+      <c r="C2" s="86"/>
+      <c r="D2" s="86"/>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="83" t="s">
         <v>76</v>
       </c>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
+      <c r="C3" s="83"/>
+      <c r="D3" s="83"/>
     </row>
     <row r="5" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="87" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="F5" s="67" t="s">
+      <c r="C5" s="87"/>
+      <c r="D5" s="87"/>
+      <c r="F5" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="G5" s="67" t="s">
+      <c r="G5" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="H5" s="67" t="s">
+      <c r="H5" s="1" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="F6" s="34" t="s">
+      <c r="F6" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="G6" s="68" t="s">
+      <c r="G6" s="54" t="s">
         <v>81</v>
       </c>
-      <c r="H6" s="17" t="s">
+      <c r="H6" s="6" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="C7" s="24" t="s">
+      <c r="C7" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="F7" s="37" t="s">
+      <c r="F7" s="26" t="s">
         <v>85</v>
       </c>
-      <c r="G7" s="69" t="s">
+      <c r="G7" s="55" t="s">
         <v>86</v>
       </c>
-      <c r="H7" s="22" t="s">
+      <c r="H7" s="11" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="8" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="C8" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="F8" s="40" t="s">
+      <c r="F8" s="29" t="s">
         <v>90</v>
       </c>
-      <c r="G8" s="70" t="s">
+      <c r="G8" s="56" t="s">
         <v>91</v>
       </c>
-      <c r="H8" s="27" t="s">
+      <c r="H8" s="16" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="10" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="87" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="F10" s="67" t="s">
+      <c r="C10" s="87"/>
+      <c r="D10" s="87"/>
+      <c r="F10" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="G10" s="67" t="s">
+      <c r="G10" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="67" t="s">
+      <c r="H10" s="1" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="11" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="34" t="s">
+      <c r="B11" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="C11" s="35" t="s">
+      <c r="C11" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="D11" s="36">
+      <c r="D11" s="25">
         <f>IF(C7="Domestico",IF(C8="Standard",40,IF(C8="Silver",80,100)),IF(C7="Condominio",IF(C8="Standard",100,IF(C8="Gold",200,IF(C8="Platinum",350,400))),IF(C8="SA",240,120)))</f>
         <v>100</v>
       </c>
-      <c r="F11" s="34" t="s">
+      <c r="F11" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="G11" s="68" t="s">
+      <c r="G11" s="54" t="s">
         <v>91</v>
       </c>
-      <c r="H11" s="17" t="s">
+      <c r="H11" s="6" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="12" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="37" t="s">
+      <c r="B12" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="C12" s="38" t="s">
+      <c r="C12" s="27" t="s">
         <v>98</v>
       </c>
-      <c r="D12" s="71">
+      <c r="D12" s="57">
         <f>IF(C7="Domestico",IF(C8="Standard",36,IF(C8="Silver",72,90)),IF(C7="Condominio",IF(C8="Standard",50,IF(C8="Gold",175,IF(C8="Platinum",200,300))),IF(C8="SA",180,60)))</f>
         <v>50</v>
       </c>
-      <c r="F12" s="37" t="s">
+      <c r="F12" s="26" t="s">
         <v>90</v>
       </c>
-      <c r="G12" s="69" t="s">
+      <c r="G12" s="55" t="s">
         <v>99</v>
       </c>
-      <c r="H12" s="22" t="s">
+      <c r="H12" s="11" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="13" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="40" t="s">
+      <c r="B13" s="29" t="s">
         <v>101</v>
       </c>
-      <c r="C13" s="72" t="str">
+      <c r="C13" s="58" t="str">
         <f>IF(C7="Domestico","non previsto",IF(C7="Condominio","€5/MWh","€2/MWh"))</f>
         <v>€5/MWh</v>
       </c>
-      <c r="D13" s="73">
+      <c r="D13" s="59">
         <f>IF(C7="Domestico",0,IF(C7="Condominio",5,2))</f>
         <v>5</v>
       </c>
-      <c r="F13" s="40" t="s">
+      <c r="F13" s="29" t="s">
         <v>89</v>
       </c>
-      <c r="G13" s="70" t="s">
+      <c r="G13" s="56" t="s">
         <v>102</v>
       </c>
-      <c r="H13" s="27" t="s">
+      <c r="H13" s="16" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="F14" s="57" t="s">
+      <c r="F14" s="44" t="s">
         <v>103</v>
       </c>
-      <c r="G14" s="74" t="s">
+      <c r="G14" s="60" t="s">
         <v>104</v>
       </c>
-      <c r="H14" s="49" t="s">
+      <c r="H14" s="36" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="15" spans="2:8" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="88" t="s">
         <v>106</v>
       </c>
-      <c r="C15" s="3"/>
-      <c r="D15" s="75">
+      <c r="C15" s="88"/>
+      <c r="D15" s="61">
         <f>D11</f>
         <v>100</v>
       </c>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="F16" s="67" t="s">
+      <c r="F16" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="G16" s="67" t="s">
+      <c r="G16" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="H16" s="67" t="s">
+      <c r="H16" s="1" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="77" t="s">
         <v>108</v>
       </c>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="F17" s="34" t="s">
+      <c r="C17" s="77"/>
+      <c r="D17" s="77"/>
+      <c r="F17" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="G17" s="68" t="s">
+      <c r="G17" s="54" t="s">
         <v>110</v>
       </c>
-      <c r="H17" s="17" t="s">
+      <c r="H17" s="6" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="18" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="45" t="s">
+      <c r="B18" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="D18" s="47">
+      <c r="D18" s="35">
         <f>ROUND(D15*0.01,2)</f>
         <v>1</v>
       </c>
-      <c r="F18" s="37" t="s">
+      <c r="F18" s="26" t="s">
         <v>112</v>
       </c>
-      <c r="G18" s="69" t="s">
+      <c r="G18" s="55" t="s">
         <v>113</v>
       </c>
-      <c r="H18" s="22" t="s">
+      <c r="H18" s="11" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="19" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="45" t="s">
+      <c r="B19" s="33" t="s">
         <v>42</v>
       </c>
-      <c r="D19" s="47">
+      <c r="D19" s="35">
         <f>ROUND(D15*0.23*0.2,2)</f>
         <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="20" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="45" t="s">
+      <c r="B20" s="33" t="s">
         <v>46</v>
       </c>
-      <c r="C20" s="46" t="str">
+      <c r="C20" s="34" t="str">
         <f>TEXT(D20/D15*100,"0.00")&amp;"% del lordo"</f>
         <v>006% del lordo</v>
       </c>
-      <c r="D20" s="47">
+      <c r="D20" s="35">
         <f>D18+D19</f>
         <v>5.6</v>
       </c>
-      <c r="F20" s="67" t="s">
+      <c r="F20" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="G20" s="76"/>
-      <c r="H20" s="67" t="s">
+      <c r="G20" s="62"/>
+      <c r="H20" s="1" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="F21" s="77" t="s">
+      <c r="F21" s="63" t="s">
         <v>117</v>
       </c>
-      <c r="H21" s="30" t="s">
+      <c r="H21" s="19" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="22" spans="2:8" ht="64.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="78" t="s">
         <v>119</v>
       </c>
-      <c r="C22" s="8"/>
-      <c r="D22" s="51">
+      <c r="C22" s="78"/>
+      <c r="D22" s="38">
         <f>D15-D20</f>
         <v>94.4</v>
       </c>
-      <c r="F22" s="60" t="s">
+      <c r="F22" s="47" t="s">
         <v>120</v>
       </c>
-      <c r="H22" s="78" t="s">
+      <c r="H22" s="64" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="23" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="F23" s="77" t="s">
+      <c r="F23" s="63" t="s">
         <v>109</v>
       </c>
-      <c r="H23" s="79" t="s">
+      <c r="H23" s="65" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="24" spans="2:8" ht="39" x14ac:dyDescent="0.2">
-      <c r="B24" s="80" t="s">
+      <c r="B24" s="66" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="25" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="F25" s="15" t="s">
+      <c r="F25" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="G25" s="81"/>
-      <c r="H25" s="15" t="s">
+      <c r="G25" s="67"/>
+      <c r="H25" s="4" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="26" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="F26" s="53" t="s">
+      <c r="F26" s="40" t="s">
         <v>55</v>
       </c>
-      <c r="H26" s="54" t="s">
+      <c r="H26" s="41" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="27" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="F27" s="53" t="s">
+      <c r="F27" s="40" t="s">
         <v>58</v>
       </c>
-      <c r="H27" s="54" t="s">
+      <c r="H27" s="41" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="28" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="F28" s="45" t="s">
+      <c r="F28" s="33" t="s">
         <v>124</v>
       </c>
-      <c r="H28" s="55" t="s">
+      <c r="H28" s="42" t="s">
         <v>61</v>
       </c>
     </row>
@@ -2427,409 +2427,409 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="89" t="s">
         <v>125</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
+      <c r="C2" s="89"/>
+      <c r="D2" s="89"/>
     </row>
     <row r="3" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="83" t="s">
         <v>126</v>
       </c>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
+      <c r="C3" s="83"/>
+      <c r="D3" s="83"/>
     </row>
     <row r="5" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="F5" s="44" t="s">
+      <c r="C5" s="77"/>
+      <c r="D5" s="77"/>
+      <c r="F5" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="G5" s="44" t="s">
+      <c r="G5" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="H5" s="44" t="s">
+      <c r="H5" s="3" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F6" s="34" t="s">
+      <c r="F6" s="23" t="s">
         <v>129</v>
       </c>
-      <c r="G6" s="82">
+      <c r="G6" s="68">
         <v>90</v>
       </c>
-      <c r="H6" s="17" t="s">
+      <c r="H6" s="6" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="C7" s="20">
+      <c r="C7" s="9">
         <v>80</v>
       </c>
-      <c r="F7" s="37" t="s">
+      <c r="F7" s="26" t="s">
         <v>132</v>
       </c>
-      <c r="G7" s="83">
+      <c r="G7" s="69">
         <v>60</v>
       </c>
-      <c r="H7" s="22" t="s">
+      <c r="H7" s="11" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="8" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="C8" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="F8" s="40" t="s">
+      <c r="F8" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="G8" s="84">
+      <c r="G8" s="70">
         <v>40</v>
       </c>
-      <c r="H8" s="27" t="s">
+      <c r="H8" s="16" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="9" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="13" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="10" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="C10" s="24" t="s">
+      <c r="C10" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="F10" s="44" t="s">
+      <c r="F10" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="G10" s="44" t="s">
+      <c r="G10" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="44" t="s">
+      <c r="H10" s="3" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="11" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="C11" s="24" t="s">
+      <c r="C11" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="F11" s="34" t="s">
+      <c r="F11" s="23" t="s">
         <v>129</v>
       </c>
-      <c r="G11" s="82">
+      <c r="G11" s="68">
         <v>150</v>
       </c>
-      <c r="H11" s="17" t="s">
+      <c r="H11" s="6" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="12" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="C12" s="24" t="s">
+      <c r="C12" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="F12" s="37" t="s">
+      <c r="F12" s="26" t="s">
         <v>132</v>
       </c>
-      <c r="G12" s="83">
+      <c r="G12" s="69">
         <v>120</v>
       </c>
-      <c r="H12" s="22" t="s">
+      <c r="H12" s="11" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="13" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F13" s="40" t="s">
+      <c r="F13" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="G13" s="84">
+      <c r="G13" s="70">
         <v>90</v>
       </c>
-      <c r="H13" s="27" t="s">
+      <c r="H13" s="16" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="14" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="77" t="s">
         <v>148</v>
       </c>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="F14" s="85" t="s">
+      <c r="C14" s="77"/>
+      <c r="D14" s="77"/>
+      <c r="F14" s="71" t="s">
         <v>149</v>
       </c>
-      <c r="G14" s="86">
+      <c r="G14" s="72">
         <v>50</v>
       </c>
-      <c r="H14" s="30" t="s">
+      <c r="H14" s="19" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="15" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="34" t="s">
+      <c r="B15" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="C15" s="35" t="s">
+      <c r="C15" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="D15" s="36">
+      <c r="D15" s="25">
         <f>IF(C8="Domestico",IF(C9="A",90,IF(C9="M",60,40)),IF(C9="A",150,IF(C9="M",120,IF(C9="B",90,50))))</f>
         <v>90</v>
       </c>
     </row>
     <row r="16" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="37" t="s">
+      <c r="B16" s="26" t="s">
         <v>151</v>
       </c>
-      <c r="C16" s="38" t="str">
+      <c r="C16" s="27" t="str">
         <f>IF(C11="Si","attivo","no")</f>
         <v>attivo</v>
       </c>
-      <c r="D16" s="71">
+      <c r="D16" s="57">
         <f>IF(C11="Si",15,0)</f>
         <v>15</v>
       </c>
-      <c r="F16" s="44" t="s">
+      <c r="F16" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="G16" s="44" t="s">
+      <c r="G16" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="H16" s="44" t="s">
+      <c r="H16" s="3" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="37" t="s">
+      <c r="B17" s="26" t="s">
         <v>155</v>
       </c>
-      <c r="C17" s="38" t="str">
+      <c r="C17" s="27" t="str">
         <f>IF(C12="Si","attivo","no")</f>
         <v>attivo</v>
       </c>
-      <c r="D17" s="71">
+      <c r="D17" s="57">
         <f>IF(C12="Si",5,0)</f>
         <v>5</v>
       </c>
-      <c r="F17" s="26" t="s">
+      <c r="F17" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="G17" s="27" t="s">
+      <c r="G17" s="16" t="s">
         <v>157</v>
       </c>
-      <c r="H17" s="84">
+      <c r="H17" s="70">
         <v>5</v>
       </c>
     </row>
     <row r="18" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="40" t="s">
+      <c r="B18" s="29" t="s">
         <v>158</v>
       </c>
-      <c r="C18" s="41" t="str">
+      <c r="C18" s="30" t="str">
         <f>IF(C7&gt;=121,"Fascia 3",IF(C7&gt;=81,"Fascia 2",IF(C7&gt;=50,"Fascia 1","Sotto soglia")))</f>
         <v>Fascia 1</v>
       </c>
-      <c r="D18" s="73">
+      <c r="D18" s="59">
         <f>IF(C7&gt;=121,15,IF(C7&gt;=81,10,IF(C7&gt;=50,5,0)))</f>
         <v>5</v>
       </c>
-      <c r="F18" s="26" t="s">
+      <c r="F18" s="15" t="s">
         <v>159</v>
       </c>
-      <c r="G18" s="27" t="s">
+      <c r="G18" s="16" t="s">
         <v>160</v>
       </c>
-      <c r="H18" s="84">
+      <c r="H18" s="70">
         <v>10</v>
       </c>
     </row>
     <row r="19" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F19" s="26" t="s">
+      <c r="F19" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="G19" s="27" t="s">
+      <c r="G19" s="16" t="s">
         <v>162</v>
       </c>
-      <c r="H19" s="84">
+      <c r="H19" s="70">
         <v>15</v>
       </c>
     </row>
     <row r="20" spans="2:8" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="90" t="s">
         <v>148</v>
       </c>
-      <c r="C20" s="1"/>
-      <c r="D20" s="87">
+      <c r="C20" s="90"/>
+      <c r="D20" s="73">
         <f>D15+D16+D17+D18</f>
         <v>115</v>
       </c>
     </row>
     <row r="21" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F21" s="44" t="s">
+      <c r="F21" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="G21" s="88"/>
-      <c r="H21" s="44" t="s">
+      <c r="G21" s="74"/>
+      <c r="H21" s="3" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="77" t="s">
         <v>163</v>
       </c>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="F22" s="53" t="s">
+      <c r="C22" s="77"/>
+      <c r="D22" s="77"/>
+      <c r="F22" s="40" t="s">
         <v>164</v>
       </c>
-      <c r="H22" s="54" t="s">
+      <c r="H22" s="41" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="23" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="45" t="s">
+      <c r="B23" s="33" t="s">
         <v>166</v>
       </c>
-      <c r="C23" s="46" t="s">
+      <c r="C23" s="34" t="s">
         <v>167</v>
       </c>
-      <c r="D23" s="47">
+      <c r="D23" s="35">
         <f>ROUND(D20*0.22,2)</f>
         <v>25.3</v>
       </c>
-      <c r="F23" s="53" t="s">
+      <c r="F23" s="40" t="s">
         <v>55</v>
       </c>
-      <c r="H23" s="54" t="s">
+      <c r="H23" s="41" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="24" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="45" t="s">
+      <c r="B24" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="C24" s="46" t="s">
+      <c r="C24" s="34" t="s">
         <v>167</v>
       </c>
-      <c r="D24" s="47">
+      <c r="D24" s="35">
         <f>ROUND(D20*0.01,2)</f>
         <v>1.1499999999999999</v>
       </c>
-      <c r="F24" s="53" t="s">
+      <c r="F24" s="40" t="s">
         <v>58</v>
       </c>
-      <c r="H24" s="54" t="s">
+      <c r="H24" s="41" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="25" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="45" t="s">
+      <c r="B25" s="33" t="s">
         <v>42</v>
       </c>
-      <c r="C25" s="46" t="s">
+      <c r="C25" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="D25" s="47">
+      <c r="D25" s="35">
         <f>ROUND(D20*0.23*0.2,2)</f>
         <v>5.29</v>
       </c>
-      <c r="F25" s="45" t="s">
+      <c r="F25" s="33" t="s">
         <v>168</v>
       </c>
-      <c r="H25" s="55" t="s">
+      <c r="H25" s="42" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="26" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="45" t="s">
+      <c r="B26" s="33" t="s">
         <v>46</v>
       </c>
-      <c r="C26" s="46" t="str">
+      <c r="C26" s="34" t="str">
         <f>TEXT(D26/D20*100,"0.00")&amp;"% del lordo"</f>
         <v>028% del lordo</v>
       </c>
-      <c r="D26" s="47">
+      <c r="D26" s="35">
         <f>D23+D24+D25</f>
         <v>31.74</v>
       </c>
     </row>
     <row r="28" spans="2:8" ht="64.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="78" t="s">
         <v>170</v>
       </c>
-      <c r="C28" s="8"/>
-      <c r="D28" s="51">
+      <c r="C28" s="78"/>
+      <c r="D28" s="38">
         <f>D20-D26</f>
         <v>83.26</v>
       </c>
     </row>
     <row r="30" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="79" t="s">
         <v>171</v>
       </c>
-      <c r="C30" s="7"/>
-      <c r="D30" s="7"/>
+      <c r="C30" s="79"/>
+      <c r="D30" s="79"/>
     </row>
     <row r="31" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="40" t="s">
+      <c r="B31" s="29" t="s">
         <v>172</v>
       </c>
-      <c r="C31" s="72" t="s">
+      <c r="C31" s="58" t="s">
         <v>173</v>
       </c>
-      <c r="D31" s="89">
+      <c r="D31" s="75">
         <f>IF(C8="Domestico",IF(C9="A",0.01,IF(C9="M",0.01,0.003)),IF(C9="A",0.004,IF(C9="M",0.003,IF(C9="B",0.002,0.0015))))</f>
         <v>0.01</v>
       </c>
     </row>
     <row r="32" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="40" t="s">
+      <c r="B32" s="29" t="s">
         <v>174</v>
       </c>
-      <c r="C32" s="72" t="s">
+      <c r="C32" s="58" t="s">
         <v>173</v>
       </c>
-      <c r="D32" s="90">
+      <c r="D32" s="76">
         <f>IF(C8="Domestico",IF(C9="A",0.05,IF(C9="M",0.05,0.02)),IF(C9="A",0.04,IF(C9="M",0.03,IF(C9="B",0.02,0.01))))</f>
         <v>0.05</v>
       </c>
     </row>
     <row r="33" spans="2:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="40" t="s">
+      <c r="B33" s="29" t="s">
         <v>175</v>
       </c>
-      <c r="C33" s="72" t="s">
+      <c r="C33" s="58" t="s">
         <v>176</v>
       </c>
-      <c r="D33" s="90">
+      <c r="D33" s="76">
         <f>IF(C8="Domestico",IF(C9="A",4,IF(C9="M",3,2)),IF(C9="A",7,IF(C9="M",6,IF(C9="B",5,0))))</f>
         <v>4</v>
       </c>
     </row>
     <row r="35" spans="2:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="80" t="s">
+      <c r="B35" s="66" t="s">
         <v>177</v>
       </c>
     </row>

</xml_diff>